<commit_message>
Refactor test cases and data loading assertions
- Updated test cases to reflect changes in case file naming conventions.
- Enhanced assertions for case properties, ensuring they match expected values.
- Introduced constants for module and case counts to improve maintainability.
- Added checks for prompt files to ensure they correspond with loaded cases.
- Improved readability and organization of test data loading logic.
</commit_message>
<xml_diff>
--- a/demo/data/prob.xlsx
+++ b/demo/data/prob.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,32 +436,72 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>身份核实</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>积分告知</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>权益介绍</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>活动推荐</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>无意愿</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>犹豫跟进</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>承诺到店</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>预约到店</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>流失风险</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>承诺到店</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>投诉处理</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>语音留言</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>已到店</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>语音留言</t>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>明确拒绝</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>通话结束</t>
         </is>
       </c>
     </row>
@@ -475,28 +515,52 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="D2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
         <v>5</v>
       </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>10</v>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>10</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>积分告知</t>
+          <t>身份核实</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -506,60 +570,108 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F3" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="G3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
         <v>5</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>无意愿</t>
+          <t>积分告知</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F4" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G4" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="H4" t="n">
         <v>15</v>
       </c>
+      <c r="I4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>流失风险</t>
+          <t>权益介绍</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -568,26 +680,50 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="G5" t="n">
         <v>15</v>
       </c>
       <c r="H5" t="n">
-        <v>15</v>
+        <v>20</v>
+      </c>
+      <c r="I5" t="n">
+        <v>20</v>
+      </c>
+      <c r="J5" t="n">
+        <v>10</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>承诺到店</t>
+          <t>活动推荐</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -599,16 +735,40 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="H6" t="n">
-        <v>10</v>
+        <v>20</v>
+      </c>
+      <c r="I6" t="n">
+        <v>25</v>
+      </c>
+      <c r="J6" t="n">
+        <v>15</v>
+      </c>
+      <c r="K6" t="n">
+        <v>10</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>10</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>已到店</t>
+          <t>无意愿</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -624,40 +784,504 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>25</v>
+      </c>
+      <c r="I7" t="n">
+        <v>10</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>20</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>15</v>
+      </c>
+      <c r="P7" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
+          <t>犹豫跟进</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>20</v>
+      </c>
+      <c r="G8" t="n">
+        <v>10</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>30</v>
+      </c>
+      <c r="J8" t="n">
+        <v>20</v>
+      </c>
+      <c r="K8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>承诺到店</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>15</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>60</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>预约到店</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>10</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>70</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>流失风险</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>30</v>
+      </c>
+      <c r="G11" t="n">
+        <v>10</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>20</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>20</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>10</v>
+      </c>
+      <c r="P11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>投诉处理</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>30</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>15</v>
+      </c>
+      <c r="I12" t="n">
+        <v>20</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>15</v>
+      </c>
+      <c r="P12" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
           <t>语音留言</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>已到店</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>明确拒绝</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>通话结束</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Update case directory structure in tasks configuration and modify related paths
</commit_message>
<xml_diff>
--- a/demo/data/prob.xlsx
+++ b/demo/data/prob.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="prob" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="prob" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,62 +441,62 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>权益介绍</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>无意愿</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>预约到店</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>承诺到店</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>积分告知</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>预约到店</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>无意愿</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>身份核实</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>身份确认</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>犹豫跟进</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>身份确认</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>身份核实</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>权益介绍</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>活动推荐</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>承诺到店</t>
-        </is>
-      </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>通话结束</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>已到店</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>明确拒绝</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>已到店</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>通话结束</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
@@ -527,31 +527,31 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
         <v>22</v>
       </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>28</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
+        <v>20</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
         <v>15</v>
-      </c>
-      <c r="M2" t="n">
-        <v>15</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="n">
-        <v>20</v>
       </c>
       <c r="P2" t="n">
         <v>0</v>
@@ -573,13 +573,13 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F3" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -591,10 +591,10 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
         <v>26</v>
-      </c>
-      <c r="L3" t="n">
-        <v>12</v>
       </c>
       <c r="M3" t="n">
         <v>12</v>
@@ -612,7 +612,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>积分告知</t>
+          <t>权益介绍</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -625,37 +625,37 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F4" t="n">
+        <v>12</v>
+      </c>
+      <c r="G4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
         <v>19</v>
       </c>
-      <c r="G4" t="n">
-        <v>19</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
+      <c r="L4" t="n">
+        <v>26</v>
+      </c>
+      <c r="M4" t="n">
         <v>12</v>
       </c>
-      <c r="K4" t="n">
-        <v>26</v>
-      </c>
-      <c r="L4" t="n">
-        <v>12</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
       <c r="N4" t="n">
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="P4" t="n">
         <v>0</v>
@@ -664,14 +664,14 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>预约到店</t>
+          <t>无意愿</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -683,7 +683,7 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -692,22 +692,22 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="N5" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="P5" t="n">
         <v>0</v>
@@ -716,17 +716,17 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>无意愿</t>
+          <t>预约到店</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -735,31 +735,31 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
         <v>20</v>
       </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>28</v>
-      </c>
-      <c r="L6" t="n">
-        <v>13</v>
-      </c>
-      <c r="M6" t="n">
-        <v>13</v>
-      </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="O6" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="P6" t="n">
         <v>0</v>
@@ -768,23 +768,23 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>犹豫跟进</t>
+          <t>承诺到店</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -799,19 +799,19 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="O7" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="P7" t="n">
         <v>0</v>
@@ -820,44 +820,44 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>身份确认</t>
+          <t>积分告知</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="M8" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -866,7 +866,7 @@
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -885,28 +885,28 @@
         <v>17</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F9" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
         <v>33</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
@@ -924,41 +924,41 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>权益介绍</t>
+          <t>身份确认</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="M10" t="n">
         <v>0</v>
@@ -967,35 +967,35 @@
         <v>0</v>
       </c>
       <c r="O10" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>活动推荐</t>
+          <t>犹豫跟进</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F11" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="G11" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -1010,13 +1010,13 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="N11" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
@@ -1028,26 +1028,26 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>承诺到店</t>
+          <t>活动推荐</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -1059,7 +1059,7 @@
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -1068,10 +1068,10 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="O12" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
@@ -1080,7 +1080,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>明确拒绝</t>
+          <t>通话结束</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1184,7 +1184,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>通话结束</t>
+          <t>明确拒绝</t>
         </is>
       </c>
       <c r="B15" t="n">

</xml_diff>

<commit_message>
feat: Update directory structure for demo data and adjust related paths in configuration and tests
</commit_message>
<xml_diff>
--- a/demo/data/prob.xlsx
+++ b/demo/data/prob.xlsx
@@ -441,44 +441,44 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>积分告知</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>无意愿</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>犹豫跟进</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>预约到店</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>身份核实</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>承诺到店</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>身份确认</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>权益介绍</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>无意愿</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>预约到店</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>承诺到店</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>积分告知</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>身份核实</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>身份确认</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>犹豫跟进</t>
-        </is>
-      </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
           <t>活动推荐</t>
@@ -491,12 +491,12 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>明确拒绝</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>已到店</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>明确拒绝</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
@@ -524,22 +524,22 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
         <v>15</v>
       </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>28</v>
@@ -548,10 +548,10 @@
         <v>20</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="O2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="P2" t="n">
         <v>0</v>
@@ -579,13 +579,13 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
         <v>12</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -600,10 +600,10 @@
         <v>12</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="O3" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
         <v>0</v>
@@ -612,7 +612,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>权益介绍</t>
+          <t>积分告知</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -628,22 +628,22 @@
         <v>19</v>
       </c>
       <c r="F4" t="n">
+        <v>19</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
         <v>12</v>
       </c>
-      <c r="G4" t="n">
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
         <v>12</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>19</v>
       </c>
       <c r="L4" t="n">
         <v>26</v>
@@ -680,22 +680,22 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
         <v>13</v>
       </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
         <v>28</v>
@@ -704,10 +704,10 @@
         <v>13</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="O5" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="P5" t="n">
         <v>0</v>
@@ -716,32 +716,32 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>预约到店</t>
+          <t>犹豫跟进</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="D6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -750,13 +750,13 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="M6" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="N6" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -768,7 +768,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>承诺到店</t>
+          <t>预约到店</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -784,7 +784,7 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -799,19 +799,19 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L7" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="N7" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="P7" t="n">
         <v>0</v>
@@ -820,26 +820,26 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>积分告知</t>
+          <t>身份核实</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E8" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -851,13 +851,13 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L8" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="M8" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -872,50 +872,50 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>身份核实</t>
+          <t>承诺到店</t>
         </is>
       </c>
       <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
         <v>8</v>
       </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="n">
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
         <v>17</v>
       </c>
-      <c r="E9" t="n">
-        <v>25</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>17</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="n">
-        <v>33</v>
-      </c>
       <c r="M9" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
@@ -934,7 +934,7 @@
         <v>9</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -946,10 +946,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>9</v>
+        <v>55</v>
       </c>
       <c r="I10" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -976,32 +976,32 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>犹豫跟进</t>
+          <t>权益介绍</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F11" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="G11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -1010,10 +1010,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="M11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
@@ -1044,7 +1044,7 @@
         <v>23</v>
       </c>
       <c r="F12" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="G12" t="n">
         <v>14</v>
@@ -1053,13 +1053,13 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -1068,10 +1068,10 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
         <v>14</v>
-      </c>
-      <c r="O12" t="n">
-        <v>0</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
@@ -1132,7 +1132,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>已到店</t>
+          <t>明确拒绝</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1184,7 +1184,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>明确拒绝</t>
+          <t>已到店</t>
         </is>
       </c>
       <c r="B15" t="n">

</xml_diff>

<commit_message>
feat: Remove ModuleDiversityAnalyzer and related configurations from analysis
</commit_message>
<xml_diff>
--- a/demo/data/prob.xlsx
+++ b/demo/data/prob.xlsx
@@ -431,67 +431,67 @@
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>流失风险</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>投诉处理</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>流失风险</t>
-        </is>
-      </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>权益介绍</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>承诺到店</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>身份核实</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>身份确认</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>积分告知</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>犹豫跟进</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>预约到店</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>活动推荐</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>无意愿</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>犹豫跟进</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>预约到店</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>身份核实</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>承诺到店</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>身份确认</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>权益介绍</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>活动推荐</t>
-        </is>
-      </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>明确拒绝</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>通话结束</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>明确拒绝</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
@@ -508,23 +508,23 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>投诉处理</t>
+          <t>流失风险</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -533,22 +533,22 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="L2" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="M2" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="N2" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -560,47 +560,47 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>流失风险</t>
+          <t>投诉处理</t>
         </is>
       </c>
       <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>22</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>28</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>15</v>
+      </c>
+      <c r="N3" t="n">
         <v>20</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="n">
-        <v>18</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>12</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
-        <v>26</v>
-      </c>
-      <c r="M3" t="n">
-        <v>12</v>
-      </c>
-      <c r="N3" t="n">
-        <v>12</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -612,7 +612,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>积分告知</t>
+          <t>权益介绍</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -625,34 +625,34 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
         <v>19</v>
       </c>
-      <c r="F4" t="n">
+      <c r="J4" t="n">
+        <v>12</v>
+      </c>
+      <c r="K4" t="n">
+        <v>26</v>
+      </c>
+      <c r="L4" t="n">
         <v>19</v>
       </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
         <v>12</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>12</v>
-      </c>
-      <c r="L4" t="n">
-        <v>26</v>
-      </c>
-      <c r="M4" t="n">
-        <v>12</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
@@ -664,14 +664,14 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>无意愿</t>
+          <t>承诺到店</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -680,7 +680,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -689,25 +689,25 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="L5" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="P5" t="n">
         <v>0</v>
@@ -716,44 +716,44 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>犹豫跟进</t>
+          <t>身份核实</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="E6" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="I6" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="L6" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="M6" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -768,11 +768,11 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>预约到店</t>
+          <t>身份确认</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -784,13 +784,13 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -799,41 +799,41 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>身份核实</t>
+          <t>积分告知</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E8" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -845,22 +845,22 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="L8" t="n">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="M8" t="n">
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
@@ -872,11 +872,11 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>承诺到店</t>
+          <t>犹豫跟进</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
@@ -885,13 +885,13 @@
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -900,22 +900,22 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="L9" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="M9" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="O9" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
@@ -924,17 +924,17 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>身份确认</t>
+          <t>预约到店</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -946,7 +946,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -958,29 +958,29 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="O10" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="P10" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>权益介绍</t>
+          <t>活动推荐</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
@@ -989,37 +989,37 @@
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F11" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="M11" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
@@ -1028,50 +1028,50 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>活动推荐</t>
+          <t>无意愿</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="C12" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="F12" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="N12" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="O12" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
@@ -1080,7 +1080,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>通话结束</t>
+          <t>明确拒绝</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1132,7 +1132,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>明确拒绝</t>
+          <t>通话结束</t>
         </is>
       </c>
       <c r="B14" t="n">

</xml_diff>